<commit_message>
Organizer is a searchable FIDE person on Norms, not free text; fix official name casing to FIDE house style
The Organizer field only ever had a plain text box for a bare FIDE ID
(no name lookup), unlike every other official — replaced with the same
FIDE-search combobox chief arbiter/deputies already use.

fide_display_name/1 was rendering "Firstname LASTNAME" (e.g. "Jorian
BURSSENS"); FIDE's actual house style is "LASTNAME, Firstname" (e.g.
"BURSSENS, Jorian") — flipped it, which also fixes IT3 B9/B18/B60ff and
FA1 B18.

ArbiterCombo's inputs also gained stable DOM ids: several instances of
the same component render side-by-side (chief arbiter, organizer,
deputies, extra arbiters), and LiveView's diffing can misattribute a
patch to the wrong sibling input without one.

Also dropped the D13 "Pairing System of a" label from the IT3 template
— it's not FIDE's own template, just one the maintainer and an arbiter
put together, and it's dead text nothing reads or writes.
</commit_message>
<xml_diff>
--- a/priv/norm_templates/IT3-TournamentReportForm.xlsx
+++ b/priv/norm_templates/IT3-TournamentReportForm.xlsx
@@ -1200,9 +1200,7 @@
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="5"/>
-      <c r="D13" s="6" t="s">
-        <v>88</v>
-      </c>
+      <c r="D13" s="6"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>

</xml_diff>